<commit_message>
Fix non-CO2 units in LEAP import
</commit_message>
<xml_diff>
--- a/outputs/leap_ippu_import/Kazakhstan_IPPU_LEAP_final_import.xlsx
+++ b/outputs/leap_ippu_import/Kazakhstan_IPPU_LEAP_final_import.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
   <si>
     <t>Area:</t>
   </si>
@@ -417,6 +417,30 @@
   </si>
   <si>
     <t>Interp(2024,27426.000000,2030,20569.500000,2050,9599.100000)</t>
+  </si>
+  <si>
+    <t>36.894000</t>
+  </si>
+  <si>
+    <t>Interp(2024,36.894000,2030,36.894000,2050,36.894000)</t>
+  </si>
+  <si>
+    <t>Interp(2024,36.894000,2030,27.670500,2050,12.912900)</t>
+  </si>
+  <si>
+    <t>Interp(2024,36.894000,2030,33.204600,2050,23.981100)</t>
+  </si>
+  <si>
+    <t>592.400000</t>
+  </si>
+  <si>
+    <t>Interp(2024,592.400000,2030,592.400000,2050,592.400000)</t>
+  </si>
+  <si>
+    <t>Interp(2024,592.400000,2030,414.680000,2050,177.720000)</t>
+  </si>
+  <si>
+    <t>Interp(2024,592.400000,2030,533.160000,2050,385.060000)</t>
   </si>
 </sst>
 </file>
@@ -2214,7 +2238,7 @@
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="3" t="s">
-        <v>91</v>
+        <v>130</v>
       </c>
       <c r="M28" s="3"/>
       <c r="N28" s="3" t="s">
@@ -2267,7 +2291,7 @@
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3" t="s">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="M29" s="3"/>
       <c r="N29" s="3" t="s">
@@ -2320,7 +2344,7 @@
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3" t="s">
-        <v>93</v>
+        <v>132</v>
       </c>
       <c r="M30" s="3"/>
       <c r="N30" s="3" t="s">
@@ -2373,7 +2397,7 @@
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="3" t="s">
-        <v>94</v>
+        <v>133</v>
       </c>
       <c r="M31" s="3"/>
       <c r="N31" s="3" t="s">
@@ -3592,7 +3616,7 @@
       </c>
       <c r="K54" s="3"/>
       <c r="L54" s="3" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="M54" s="3"/>
       <c r="N54" s="3" t="s">
@@ -3698,7 +3722,7 @@
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="3" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="M56" s="3"/>
       <c r="N56" s="3" t="s">
@@ -3751,7 +3775,7 @@
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="3" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="M57" s="3"/>
       <c r="N57" s="3" t="s">
@@ -3804,7 +3828,7 @@
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="3" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="M58" s="3"/>
       <c r="N58" s="3" t="s">
@@ -3857,7 +3881,7 @@
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="3" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
       <c r="M59" s="3"/>
       <c r="N59" s="3" t="s">
@@ -4016,7 +4040,7 @@
       </c>
       <c r="K62" s="3"/>
       <c r="L62" s="3" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="M62" s="3"/>
       <c r="N62" s="3" t="s">

</xml_diff>

<commit_message>
Correct LEAP import units and calculation wording
Write the ferroalloy CH4 and nitric-acid N2O branches in kilograms, the
unit of the LEAP template, and move the scenario parameters to
data/metadata/leap_scenario_parameters.csv. The import script now stops
if a template unit differs from the parameter file.

In the conference documents, describe the results as computed with
LEAP's deterministic Interp() expressions and reproduced in Python, and
the 2024 base year as a 2023 inventory proxy. Ignore Python bytecode
and local session notes.
</commit_message>
<xml_diff>
--- a/outputs/leap_ippu_import/Kazakhstan_IPPU_LEAP_final_import.xlsx
+++ b/outputs/leap_ippu_import/Kazakhstan_IPPU_LEAP_final_import.xlsx
@@ -2238,7 +2238,7 @@
       </c>
       <c r="K28" s="3"/>
       <c r="L28" s="3" t="s">
-        <v>130</v>
+        <v>91</v>
       </c>
       <c r="M28" s="3"/>
       <c r="N28" s="3" t="s">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="K29" s="3"/>
       <c r="L29" s="3" t="s">
-        <v>131</v>
+        <v>92</v>
       </c>
       <c r="M29" s="3"/>
       <c r="N29" s="3" t="s">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="K30" s="3"/>
       <c r="L30" s="3" t="s">
-        <v>132</v>
+        <v>93</v>
       </c>
       <c r="M30" s="3"/>
       <c r="N30" s="3" t="s">
@@ -2397,7 +2397,7 @@
       </c>
       <c r="K31" s="3"/>
       <c r="L31" s="3" t="s">
-        <v>133</v>
+        <v>94</v>
       </c>
       <c r="M31" s="3"/>
       <c r="N31" s="3" t="s">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="K56" s="3"/>
       <c r="L56" s="3" t="s">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="M56" s="3"/>
       <c r="N56" s="3" t="s">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="K57" s="3"/>
       <c r="L57" s="3" t="s">
-        <v>135</v>
+        <v>120</v>
       </c>
       <c r="M57" s="3"/>
       <c r="N57" s="3" t="s">
@@ -3828,7 +3828,7 @@
       </c>
       <c r="K58" s="3"/>
       <c r="L58" s="3" t="s">
-        <v>136</v>
+        <v>121</v>
       </c>
       <c r="M58" s="3"/>
       <c r="N58" s="3" t="s">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="K59" s="3"/>
       <c r="L59" s="3" t="s">
-        <v>137</v>
+        <v>122</v>
       </c>
       <c r="M59" s="3"/>
       <c r="N59" s="3" t="s">

</xml_diff>